<commit_message>
sim2 v6: refresh downloadable datasets to the v6 serial-date files
public/sim2-data Round1_RawFeed.xlsx and Round3_NewMonth_RawFeed.xlsx were the old
v1 dataset (wrong content — students would compute the wrong numbers). Replaced with
the v6 source files (verified to yield 62,667 / 1,381,546 / 270 / Notebook Set 35 /
April 90). Removed the unused v1 master + prior-quarter files.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/sim2-data/Round1_RawFeed.xlsx
+++ b/public/sim2-data/Round1_RawFeed.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>21-01-2026-Wireless Mouse-799-3</t>
+          <t>46043-Wireless Mouse-799-3</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05-03-2026-Laptop Charger-1299-5</t>
+          <t>46086-Laptop Charger-1299-5</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -469,7 +469,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>02-01-2026-Laptop Charger-1299-2</t>
+          <t>46024-Laptop Charger-1299-2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -484,7 +484,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18-01-2026-Webcam HD-2199-4</t>
+          <t>46040-Webcam HD-2199-4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -499,7 +499,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19-02-2026-Wireless Mouse-799-2</t>
+          <t>46072-Wireless Mouse-799-2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11-02-2026-Bluetooth Speaker-1899-2</t>
+          <t>46064-Bluetooth Speaker-1899-2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03-02-2026-Laptop Charger-1299-3</t>
+          <t>46056-Laptop Charger-1299-3</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>26-01-2026-Whiteboard-1599-5</t>
+          <t>46048-Whiteboard-1599-5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>03-03-2026-Desk Lamp-699-5</t>
+          <t>46084-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>23-01-2026-Wireless Mouse-799-2</t>
+          <t>46045-Wireless Mouse-799-2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28-01-2026-Laptop Charger-1299-4</t>
+          <t>46050-Laptop Charger-1299-4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21-02-2026-Bluetooth Speaker-1899-3</t>
+          <t>46074-Bluetooth Speaker-1899-3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>22-02-2026-Laptop Charger-1299-5</t>
+          <t>46075-Laptop Charger-1299-5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>18-03-2026-USB-C Hub-999-2</t>
+          <t>46099-USB-C Hub-999-2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09-03-2026-Webcam HD-2199-2</t>
+          <t>46090-Webcam HD-2199-2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>27-01-2026-USB-C Hub-999-1</t>
+          <t>46049-USB-C Hub-999-1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09-01-2026-USB-C Hub-999-5</t>
+          <t>46031-USB-C Hub-999-5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07-03-2026-Whiteboard-1599-4</t>
+          <t>46088-Whiteboard-1599-4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05-02-2026-Bluetooth Speaker-1899-2</t>
+          <t>46058-Bluetooth Speaker-1899-2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>24-03-2026-Notebook Set-249-5</t>
+          <t>46105-Notebook Set-249-5</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08-01-2026-Webcam HD-2199-4</t>
+          <t>46030-Webcam HD-2199-4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28-01-2026-Bluetooth Speaker-1899-2</t>
+          <t>46050-Bluetooth Speaker-1899-2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>20-01-2026-Notebook Set-249-4</t>
+          <t>46042-Notebook Set-249-4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>17-02-2026-Webcam HD-2199-1</t>
+          <t>46070-Webcam HD-2199-1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>22-03-2026-Desk Lamp-699-3</t>
+          <t>46103-Desk Lamp-699-3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14-01-2026-Whiteboard-1599-1</t>
+          <t>46036-Whiteboard-1599-1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>17-01-2026-Webcam HD-2199-1</t>
+          <t>46039-Webcam HD-2199-1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>27-03-2026-Webcam HD-2199-5</t>
+          <t>46108-Webcam HD-2199-5</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>12-01-2026-Webcam HD-2199-5</t>
+          <t>46034-Webcam HD-2199-5</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>16-01-2026-Laptop Charger-1299-3</t>
+          <t>46038-Laptop Charger-1299-3</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>02-01-2026-Mechanical Keyboard-3299-1</t>
+          <t>46024-Mechanical Keyboard-3299-1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27-01-2026-Webcam HD-2199-2</t>
+          <t>46049-Webcam HD-2199-2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>18-01-2026-Desk Lamp-699-5</t>
+          <t>46040-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07-03-2026-USB-C Hub-999-3</t>
+          <t>46088-USB-C Hub-999-3</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15-03-2026-Whiteboard-1599-1</t>
+          <t>46096-Whiteboard-1599-1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>03-02-2026-Wireless Mouse-799-5</t>
+          <t>46056-Wireless Mouse-799-5</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>19-01-2026-Wireless Mouse-799-1</t>
+          <t>46041-Wireless Mouse-799-1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08-01-2026-Wireless Mouse-799-3</t>
+          <t>46030-Wireless Mouse-799-3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09-03-2026-Whiteboard-1599-2</t>
+          <t>46090-Whiteboard-1599-2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>24-03-2026-Mechanical Keyboard-3299-4</t>
+          <t>46105-Mechanical Keyboard-3299-4</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26-02-2026-USB-C Hub-999-1</t>
+          <t>46079-USB-C Hub-999-1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>12-02-2026-Notebook Set-249-4</t>
+          <t>46065-Notebook Set-249-4</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>22-03-2026-Laptop Charger-1299-1</t>
+          <t>46103-Laptop Charger-1299-1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>26-01-2026-USB-C Hub-999-2</t>
+          <t>46048-USB-C Hub-999-2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>05-02-2026-Bluetooth Speaker-1899-3</t>
+          <t>46058-Bluetooth Speaker-1899-3</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28-01-2026-Whiteboard-1599-5</t>
+          <t>46050-Whiteboard-1599-5</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>21-03-2026-Wireless Mouse-799-1</t>
+          <t>46102-Wireless Mouse-799-1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>14-02-2026-Whiteboard-1599-2</t>
+          <t>46067-Whiteboard-1599-2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>06-02-2026-Wireless Mouse-799-4</t>
+          <t>46059-Wireless Mouse-799-4</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10-02-2026-Webcam HD-2199-4</t>
+          <t>46063-Webcam HD-2199-4</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>10-01-2026-Wireless Mouse-799-5</t>
+          <t>46032-Wireless Mouse-799-5</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>24-02-2026-Wireless Mouse-799-1</t>
+          <t>46077-Wireless Mouse-799-1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>17-03-2026-Bluetooth Speaker-1899-1</t>
+          <t>46098-Bluetooth Speaker-1899-1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>28-01-2026-Laptop Charger-1299-5</t>
+          <t>46050-Laptop Charger-1299-5</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>13-01-2026-Mechanical Keyboard-3299-2</t>
+          <t>46035-Mechanical Keyboard-3299-2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>20-01-2026-Notebook Set-249-5</t>
+          <t>46042-Notebook Set-249-5</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09-01-2026-Office Chair-6499-2</t>
+          <t>46031-Office Chair-6499-2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>05-03-2026-Desk Lamp-699-4</t>
+          <t>46086-Desk Lamp-699-4</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>01-02-2026-Mechanical Keyboard-3299-5</t>
+          <t>46054-Mechanical Keyboard-3299-5</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>18-01-2026-Webcam HD-2199-3</t>
+          <t>46040-Webcam HD-2199-3</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>03-01-2026-Office Chair-6499-3</t>
+          <t>46025-Office Chair-6499-3</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27-03-2026-Desk Lamp-699-5</t>
+          <t>46108-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>22-03-2026-Desk Lamp-699-1</t>
+          <t>46103-Desk Lamp-699-1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04-01-2026-Webcam HD-2199-2</t>
+          <t>46026-Webcam HD-2199-2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>20-01-2026-Office Chair-6499-2</t>
+          <t>46042-Office Chair-6499-2</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>17-02-2026-Desk Lamp-699-1</t>
+          <t>46070-Desk Lamp-699-1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>27-02-2026-Wireless Mouse-799-1</t>
+          <t>46080-Wireless Mouse-799-1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>21-02-2026-Bluetooth Speaker-1899-4</t>
+          <t>46074-Bluetooth Speaker-1899-4</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>18-01-2026-Laptop Charger-1299-1</t>
+          <t>46040-Laptop Charger-1299-1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>18-01-2026-Office Chair-6499-5</t>
+          <t>46040-Office Chair-6499-5</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>14-01-2026-Wireless Mouse-799-3</t>
+          <t>46036-Wireless Mouse-799-3</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>12-01-2026-USB-C Hub-999-1</t>
+          <t>46034-USB-C Hub-999-1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>20-03-2026-Bluetooth Speaker-1899-2</t>
+          <t>46101-Bluetooth Speaker-1899-2</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>14-01-2026-Bluetooth Speaker-1899-3</t>
+          <t>46036-Bluetooth Speaker-1899-3</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09-01-2026-Laptop Charger-1299-4</t>
+          <t>46031-Laptop Charger-1299-4</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08-01-2026-Whiteboard-1599-3</t>
+          <t>46030-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08-01-2026-USB-C Hub-999-4</t>
+          <t>46030-USB-C Hub-999-4</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>28-01-2026-Desk Lamp-699-3</t>
+          <t>46050-Desk Lamp-699-3</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>22-03-2026-Office Chair-6499-1</t>
+          <t>46103-Office Chair-6499-1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>06-03-2026-Desk Lamp-699-1</t>
+          <t>46087-Desk Lamp-699-1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>12-03-2026-Office Chair-6499-4</t>
+          <t>46093-Office Chair-6499-4</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>13-03-2026-USB-C Hub-999-3</t>
+          <t>46094-USB-C Hub-999-3</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01-03-2026-Webcam HD-2199-2</t>
+          <t>46082-Webcam HD-2199-2</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>03-03-2026-Office Chair-6499-5</t>
+          <t>46084-Office Chair-6499-5</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>24-02-2026-Webcam HD-2199-3</t>
+          <t>46077-Webcam HD-2199-3</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>11-02-2026-Desk Lamp-699-5</t>
+          <t>46064-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>14-03-2026-Notebook Set-249-2</t>
+          <t>46095-Notebook Set-249-2</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>13-03-2026-Wireless Mouse-799-3</t>
+          <t>46094-Wireless Mouse-799-3</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>14-03-2026-Mechanical Keyboard-3299-3</t>
+          <t>46095-Mechanical Keyboard-3299-3</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>15-03-2026-USB-C Hub-999-5</t>
+          <t>46096-USB-C Hub-999-5</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>22-01-2026-Desk Lamp-699-5</t>
+          <t>46044-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>03-01-2026-Desk Lamp-699-2</t>
+          <t>46025-Desk Lamp-699-2</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>01-01-2026-USB-C Hub-999-4</t>
+          <t>46023-USB-C Hub-999-4</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>15-02-2026-Mechanical Keyboard-3299-2</t>
+          <t>46068-Mechanical Keyboard-3299-2</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>16-02-2026-USB-C Hub-999-2</t>
+          <t>46069-USB-C Hub-999-2</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>25-01-2026-Notebook Set-249-2</t>
+          <t>46047-Notebook Set-249-2</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>02-03-2026-USB-C Hub-999-1</t>
+          <t>46083-USB-C Hub-999-1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>26-02-2026-Webcam HD-2199-5</t>
+          <t>46079-Webcam HD-2199-5</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>25-02-2026-Mechanical Keyboard-3299-5</t>
+          <t>46078-Mechanical Keyboard-3299-5</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>06-03-2026-Whiteboard-1599-4</t>
+          <t>46087-Whiteboard-1599-4</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>27-03-2026-Desk Lamp-699-5</t>
+          <t>46108-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>09-02-2026-Laptop Charger-1299-3</t>
+          <t>46062-Laptop Charger-1299-3</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11-02-2026-Webcam HD-2199-1</t>
+          <t>46064-Webcam HD-2199-1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>08-02-2026-Bluetooth Speaker-1899-2</t>
+          <t>46061-Bluetooth Speaker-1899-2</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>14-02-2026-Webcam HD-2199-4</t>
+          <t>46067-Webcam HD-2199-4</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>07-02-2026-Notebook Set-249-5</t>
+          <t>46060-Notebook Set-249-5</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>28-03-2026-Notebook Set-249-4</t>
+          <t>46109-Notebook Set-249-4</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10-02-2026-Notebook Set-249-5</t>
+          <t>46063-Notebook Set-249-5</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>16-01-2026-Desk Lamp-699-4</t>
+          <t>46038-Desk Lamp-699-4</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>13-02-2026-Notebook Set-249-2</t>
+          <t>46066-Notebook Set-249-2</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>20-03-2026-Wireless Mouse-799-4</t>
+          <t>46101-Wireless Mouse-799-4</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>03-03-2026-Notebook Set-249-2</t>
+          <t>46084-Notebook Set-249-2</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>02-02-2026-Notebook Set-249-3</t>
+          <t>46055-Notebook Set-249-3</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11-02-2026-Notebook Set-249-3</t>
+          <t>46064-Notebook Set-249-3</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>27-01-2026-Whiteboard-1599-1</t>
+          <t>46049-Whiteboard-1599-1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12-01-2026-Laptop Charger-1299-1</t>
+          <t>46034-Laptop Charger-1299-1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>07-01-2026-Mechanical Keyboard-3299-2</t>
+          <t>46029-Mechanical Keyboard-3299-2</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>16-03-2026-Laptop Charger-1299-5</t>
+          <t>46097-Laptop Charger-1299-5</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>23-02-2026-Office Chair-6499-2</t>
+          <t>46076-Office Chair-6499-2</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>25-01-2026-Desk Lamp-699-1</t>
+          <t>46047-Desk Lamp-699-1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10-03-2026-Notebook Set-249-4</t>
+          <t>46091-Notebook Set-249-4</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>03-03-2026-USB-C Hub-999-1</t>
+          <t>46084-USB-C Hub-999-1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>28-03-2026-Mechanical Keyboard-3299-1</t>
+          <t>46109-Mechanical Keyboard-3299-1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12-03-2026-Notebook Set-249-3</t>
+          <t>46093-Notebook Set-249-3</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>01-02-2026-Whiteboard-1599-1</t>
+          <t>46054-Whiteboard-1599-1</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>21-02-2026-Bluetooth Speaker-1899-4</t>
+          <t>46074-Bluetooth Speaker-1899-4</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>20-03-2026-Whiteboard-1599-4</t>
+          <t>46101-Whiteboard-1599-4</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>11-01-2026-Laptop Charger-1299-3</t>
+          <t>46033-Laptop Charger-1299-3</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>25-02-2026-Mechanical Keyboard-3299-5</t>
+          <t>46078-Mechanical Keyboard-3299-5</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11-01-2026-Whiteboard-1599-3</t>
+          <t>46033-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>07-02-2026-Desk Lamp-699-3</t>
+          <t>46060-Desk Lamp-699-3</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>18-01-2026-Webcam HD-2199-2</t>
+          <t>46040-Webcam HD-2199-2</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>24-02-2026-Whiteboard-1599-5</t>
+          <t>46077-Whiteboard-1599-5</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>21-03-2026-Whiteboard-1599-4</t>
+          <t>46102-Whiteboard-1599-4</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10-01-2026-Notebook Set-249-2</t>
+          <t>46032-Notebook Set-249-2</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>16-03-2026-Webcam HD-2199-3</t>
+          <t>46097-Webcam HD-2199-3</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>12-03-2026-Whiteboard-1599-3</t>
+          <t>46093-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>08-01-2026-USB-C Hub-999-3</t>
+          <t>46030-USB-C Hub-999-3</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>07-01-2026-Whiteboard-1599-3</t>
+          <t>46029-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04-01-2026-Desk Lamp-699-2</t>
+          <t>46026-Desk Lamp-699-2</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>10-01-2026-Webcam HD-2199-2</t>
+          <t>46032-Webcam HD-2199-2</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>02-03-2026-Desk Lamp-699-2</t>
+          <t>46083-Desk Lamp-699-2</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>04-01-2026-Mechanical Keyboard-3299-3</t>
+          <t>46026-Mechanical Keyboard-3299-3</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>15-02-2026-Bluetooth Speaker-1899-1</t>
+          <t>46068-Bluetooth Speaker-1899-1</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>04-01-2026-Notebook Set-249-4</t>
+          <t>46026-Notebook Set-249-4</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>05-01-2026-Mechanical Keyboard-3299-3</t>
+          <t>46027-Mechanical Keyboard-3299-3</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>04-03-2026-Notebook Set-249-5</t>
+          <t>46085-Notebook Set-249-5</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>25-03-2026-Notebook Set-249-4</t>
+          <t>46106-Notebook Set-249-4</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>28-03-2026-Notebook Set-249-3</t>
+          <t>46109-Notebook Set-249-3</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>20-03-2026-Laptop Charger-1299-2</t>
+          <t>46101-Laptop Charger-1299-2</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>09-03-2026-Laptop Charger-1299-2</t>
+          <t>46090-Laptop Charger-1299-2</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>18-01-2026-Bluetooth Speaker-1899-1</t>
+          <t>46040-Bluetooth Speaker-1899-1</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>23-03-2026-Whiteboard-1599-3</t>
+          <t>46104-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>10-03-2026-Desk Lamp-699-4</t>
+          <t>46091-Desk Lamp-699-4</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>09-03-2026-Mechanical Keyboard-3299-2</t>
+          <t>46090-Mechanical Keyboard-3299-2</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>18-01-2026-Bluetooth Speaker-1899-3</t>
+          <t>46040-Bluetooth Speaker-1899-3</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>02-01-2026-Desk Lamp-699-5</t>
+          <t>46024-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>15-01-2026-Whiteboard-1599-3</t>
+          <t>46037-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>09-03-2026-Webcam HD-2199-4</t>
+          <t>46090-Webcam HD-2199-4</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>20-01-2026-Notebook Set-249-3</t>
+          <t>46042-Notebook Set-249-3</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01-01-2026-USB-C Hub-999-5</t>
+          <t>46023-USB-C Hub-999-5</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>25-03-2026-Desk Lamp-699-5</t>
+          <t>46106-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>16-03-2026-Whiteboard-1599-3</t>
+          <t>46097-Whiteboard-1599-3</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>21-02-2026-Laptop Charger-1299-4</t>
+          <t>46074-Laptop Charger-1299-4</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>11-02-2026-Laptop Charger-1299-2</t>
+          <t>46064-Laptop Charger-1299-2</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>23-02-2026-Desk Lamp-699-4</t>
+          <t>46076-Desk Lamp-699-4</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15-01-2026-Office Chair-6499-3</t>
+          <t>46037-Office Chair-6499-3</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>25-02-2026-Webcam HD-2199-1</t>
+          <t>46078-Webcam HD-2199-1</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>14-01-2026-USB-C Hub-999-5</t>
+          <t>46036-USB-C Hub-999-5</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>21-02-2026-Wireless Mouse-799-2</t>
+          <t>46074-Wireless Mouse-799-2</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>10-02-2026-Whiteboard-1599-1</t>
+          <t>46063-Whiteboard-1599-1</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>23-01-2026-Desk Lamp-699-5</t>
+          <t>46045-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>03-01-2026-Laptop Charger-1299-4</t>
+          <t>46025-Laptop Charger-1299-4</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>16-03-2026-Desk Lamp-699-5</t>
+          <t>46097-Desk Lamp-699-5</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>14-02-2026-Whiteboard-1599-2</t>
+          <t>46067-Whiteboard-1599-2</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>13-01-2026-Mechanical Keyboard-3299-5</t>
+          <t>46035-Mechanical Keyboard-3299-5</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>28-01-2026-Desk Lamp-699-4</t>
+          <t>46050-Desk Lamp-699-4</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>27-01-2026-Desk Lamp-699-3</t>
+          <t>46049-Desk Lamp-699-3</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>28-01-2026-Whiteboard-1599-5</t>
+          <t>46050-Whiteboard-1599-5</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>11-03-2026-Webcam HD-2199-4</t>
+          <t>46092-Webcam HD-2199-4</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">

</xml_diff>